<commit_message>
Recolor source workbook to Inbound palette + clean filler descriptions
- GEO-AEO-Checklist-v5.xlsx recolored to Inbound (navy→teal, blue→coral,
  priority scale harmonized) via raw OOXML edit, preserving inline-string
  structure / dropdowns / frozen panes.
- Replaced 173 generic placeholder Detay descriptions in E-Ticaret
  ("İlgili bilgi veya element eklenmeliydi." etc.) with concise, accurate
  Turkish GEO/SEO descriptions tailored to each subtask (scripts/clean_and_recolor.py).
- Source template is now pre-recolored, so the export engine reuses styles.xml
  verbatim (dropped the runtime recolor) — export stays Inbound + byte-identical.
- Regenerated checklist.json.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/GEO-AEO-Checklist-v5.xlsx
+++ b/public/GEO-AEO-Checklist-v5.xlsx
@@ -211,7 +211,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FF1F3864"/>
+      <color rgb="FF10332F"/>
       <sz val="10"/>
     </font>
     <font>
@@ -423,62 +423,62 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
-        <bgColor rgb="FF1F3864"/>
+        <fgColor rgb="FF10332F"/>
+        <bgColor rgb="FF10332F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF0F0F0"/>
-        <bgColor rgb="FFF0F0F0"/>
+        <fgColor rgb="FFF4F2EE"/>
+        <bgColor rgb="FFF4F2EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
-        <bgColor rgb="FF1F4E79"/>
+        <fgColor rgb="FF1A4238"/>
+        <bgColor rgb="FF1A4238"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2E75B6"/>
-        <bgColor rgb="FF2E75B6"/>
+        <fgColor rgb="FFFF7B52"/>
+        <bgColor rgb="FFFF7B52"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F0FE"/>
-        <bgColor rgb="FFE8F0FE"/>
+        <fgColor rgb="FFFFE3D8"/>
+        <bgColor rgb="FFFFE3D8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF6B6B"/>
-        <bgColor rgb="FFFF6B6B"/>
+        <fgColor rgb="FFE5534D"/>
+        <bgColor rgb="FFE5534D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFF4F2EE"/>
+        <bgColor rgb="FFF4F2EE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFB347"/>
-        <bgColor rgb="FFFFB347"/>
+        <fgColor rgb="FFF5A623"/>
+        <bgColor rgb="FFF5A623"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE066"/>
-        <bgColor rgb="FFFFE066"/>
+        <fgColor rgb="FFFAD46B"/>
+        <bgColor rgb="FFFAD46B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF77DD77"/>
-        <bgColor rgb="FF77DD77"/>
+        <fgColor rgb="FF8FD3A6"/>
+        <bgColor rgb="FF8FD3A6"/>
       </patternFill>
     </fill>
     <fill>
@@ -4066,7 +4066,7 @@
       </c>
       <c r="F71" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Ürün feed'i Bing Merchant Center formatına uygun hazırlanır ve gönderilerek Bing alışveriş sonuçlarında görünürlük sağlanır.</t>
         </is>
       </c>
       <c r="G71" s="137" t="n"/>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="F72" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>İşletme bilgileri Bing Places for Business'ta doğrulanır; NAP tutarlılığı korunarak yerel görünürlük artırılır.</t>
         </is>
       </c>
       <c r="G72" s="137" t="n"/>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="F74" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Sitemap'teki kırık, 404 veren, noindex veya yönlendirilen URL'ler ile orphan sayfalar tespit edilip temizlenir.</t>
         </is>
       </c>
       <c r="G74" s="137" t="n"/>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="F76" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Sitemap ürün, kategori ve blog gibi türlere bölünerek indexleme takibi ve crawl önceliklendirmesi kolaylaştırılır.</t>
         </is>
       </c>
       <c r="G76" s="137" t="n"/>
@@ -4370,7 +4370,7 @@
       </c>
       <c r="F79" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Mevcut iç link yapısı çıkarılarak orphan sayfalar, zayıf bağlantılı önemli sayfalar ve link derinliği analiz edilir.</t>
         </is>
       </c>
       <c r="G79" s="137" t="n"/>
@@ -4438,7 +4438,7 @@
       </c>
       <c r="F81" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Pillar ve cluster sayfaları arasında konu bütünlüğünü güçlendiren iç link planı oluşturulur.</t>
         </is>
       </c>
       <c r="G81" s="137" t="n"/>
@@ -4608,7 +4608,7 @@
       </c>
       <c r="F86" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>name, price, availability, brand ve aggregateRating alanlarını içeren tekrar kullanılabilir Product JSON-LD şablonu hazırlanır.</t>
         </is>
       </c>
       <c r="G86" s="137" t="n"/>
@@ -4828,7 +4828,7 @@
       </c>
       <c r="F92" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Ürün sayfalarındaki mevcut soru-cevap içerikleri taranarak FAQ schema'ya uygun bölümler belirlenir.</t>
         </is>
       </c>
       <c r="G92" s="137" t="n"/>
@@ -4862,7 +4862,7 @@
       </c>
       <c r="F93" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Soru-cevap çiftlerini içeren standart FAQPage JSON-LD şablonu hazırlanarak ürün sayfalarına uygulamaya hazır hale getirilir.</t>
         </is>
       </c>
       <c r="G93" s="137" t="n"/>
@@ -4896,7 +4896,7 @@
       </c>
       <c r="F94" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Her ürün için kullanıcıların en sık sorduğu en az 3-5 soru-cevap eklenir ve FAQ schema ile işaretlenir.</t>
         </is>
       </c>
       <c r="G94" s="137" t="n"/>
@@ -5014,7 +5014,7 @@
       </c>
       <c r="F97" s="137" t="inlineStr">
         <is>
-          <t>Veri analiz yapılmalı, insight'lar çıkarılmalıydı.</t>
+          <t>People Also Ask, forum ve müşteri destek verilerinden kategoriye özgü en yaygın sorular derlenir.</t>
         </is>
       </c>
       <c r="G97" s="137" t="n"/>
@@ -5082,7 +5082,7 @@
       </c>
       <c r="F99" s="137" t="inlineStr">
         <is>
-          <t>Action'lar implement edilmeliydi, sonuçlar measured edilmeliydi.</t>
+          <t>Hazırlanan soru-cevaplar kategori sayfalarına eklenir ve FAQPage schema ile işaretlenir.</t>
         </is>
       </c>
       <c r="G99" s="137" t="n"/>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="F102" s="137" t="inlineStr">
         <is>
-          <t>Best option research sonrası seçilmeliydi.</t>
+          <t>GSC verisine göre en çok trafik alan blog yazıları, FAQ schema önceliği için listelenir.</t>
         </is>
       </c>
       <c r="G102" s="137" t="n"/>
@@ -5268,7 +5268,7 @@
       </c>
       <c r="F104" s="137" t="inlineStr">
         <is>
-          <t>Action'lar implement edilmeliydi, sonuçlar measured edilmeliydi.</t>
+          <t>Seçilen blog yazılarındaki soru-cevap bölümleri FAQPage schema ile işaretlenir.</t>
         </is>
       </c>
       <c r="G104" s="137" t="n"/>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="F105" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Blog şablonuna standart bir SSS bölümü eklenerek her yeni yazıda FAQ schema'nın tutarlı kullanımı sağlanır.</t>
         </is>
       </c>
       <c r="G105" s="137" t="n"/>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="F107" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Kurulum, kullanım ve bakım gibi adımlı anlatıma uygun içerikler HowTo schema için belirlenir.</t>
         </is>
       </c>
       <c r="G107" s="137" t="n"/>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="F108" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>step, tool, supply ve image alanlarını içeren HowTo JSON-LD şablonu hazırlanır.</t>
         </is>
       </c>
       <c r="G108" s="137" t="n"/>
@@ -5454,7 +5454,7 @@
       </c>
       <c r="F109" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Uygun rehber içeriklere HowTo schema eklenir ve Rich Results Test ile doğrulanır.</t>
         </is>
       </c>
       <c r="G109" s="137" t="n"/>
@@ -5606,7 +5606,7 @@
       </c>
       <c r="F113" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Kategori ve listeleme sayfaları için ürün sıralamasını yansıtan ItemList JSON-LD otomatik üretilir.</t>
         </is>
       </c>
       <c r="G113" s="137" t="n"/>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="F117" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Mevcut breadcrumb yapısının site hiyerarşisiyle uyumu ve tüm şablonlarda tutarlılığı kontrol edilir.</t>
         </is>
       </c>
       <c r="G117" s="137" t="n"/>
@@ -5792,7 +5792,7 @@
       </c>
       <c r="F118" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Sayfa hiyerarşisini yansıtan BreadcrumbList JSON-LD şablonu hazırlanır.</t>
         </is>
       </c>
       <c r="G118" s="137" t="n"/>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="F119" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>BreadcrumbList schema CMS'e entegre edilerek tüm sayfalarda otomatik üretilir.</t>
         </is>
       </c>
       <c r="G119" s="137" t="n"/>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="F122" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Mevcut yorum ve puanlama sistemi incelenerek Review/AggregateRating schema için veri kaynağı belirlenir.</t>
         </is>
       </c>
       <c r="G122" s="137" t="n"/>
@@ -5978,7 +5978,7 @@
       </c>
       <c r="F123" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Gerçek müşteri yorumları ve ortalama puan Review ve AggregateRating JSON-LD ile işaretlenir.</t>
         </is>
       </c>
       <c r="G123" s="137" t="n"/>
@@ -6130,7 +6130,7 @@
       </c>
       <c r="F127" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>name, url, logo, sameAs ve contactPoint alanlarını içeren Organization JSON-LD hazırlanır.</t>
         </is>
       </c>
       <c r="G127" s="137" t="n"/>
@@ -6164,7 +6164,7 @@
       </c>
       <c r="F128" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Yazar adı, görseli, uzmanlık alanı ve sosyal profillerini içeren Person JSON-LD hazırlanır.</t>
         </is>
       </c>
       <c r="G128" s="137" t="n"/>
@@ -6198,7 +6198,7 @@
       </c>
       <c r="F129" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Organization schema ana sayfaya eklenerek markanın kurumsal kimliği AI ve aramaya net şekilde tanıtılır.</t>
         </is>
       </c>
       <c r="G129" s="137" t="n"/>
@@ -6232,7 +6232,7 @@
       </c>
       <c r="F130" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Blog yazılarına Article schema ve yazarı bağlayan author (Person) referansı eklenir.</t>
         </is>
       </c>
       <c r="G130" s="137" t="n"/>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="F133" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Tanım, hedef kitle, fayda ve özellikleri kapsayan GEO uyumlu ürün açıklaması şablonu hazırlanır.</t>
         </is>
       </c>
       <c r="G133" s="137" t="n"/>
@@ -6368,7 +6368,7 @@
       </c>
       <c r="F134" s="137" t="inlineStr">
         <is>
-          <t>Action'lar implement edilmeliydi, sonuçlar measured edilmeliydi.</t>
+          <t>Açıklamanın ilk cümlesinde ürün tanımı, hedef kitle ve ana fayda net şekilde verilir.</t>
         </is>
       </c>
       <c r="G134" s="137" t="n"/>
@@ -6436,7 +6436,7 @@
       </c>
       <c r="F136" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Her açıklamaya AI tarafından alıntılanmaya uygun, bağımsız ve net cümleler eklenir.</t>
         </is>
       </c>
       <c r="G136" s="137" t="n"/>
@@ -6554,7 +6554,7 @@
       </c>
       <c r="F139" s="137" t="inlineStr">
         <is>
-          <t>Best option research sonrası seçilmeliydi.</t>
+          <t>GSC trafiğine göre yanıt öncelikli formata dönüştürülecek en yüksek trafikli 30 sayfa seçilir.</t>
         </is>
       </c>
       <c r="G139" s="137" t="n"/>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="F140" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Her sayfanın veya bölümün başına kullanıcının sorusunu doğrudan yanıtlayan kısa bir özet paragraf eklenir.</t>
         </is>
       </c>
       <c r="G140" s="137" t="n"/>
@@ -6808,7 +6808,7 @@
       </c>
       <c r="F146" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Kategori sayfalarına o kategoriye özgü soru-cevap bölümü eklenerek içerik derinliği artırılır.</t>
         </is>
       </c>
       <c r="G146" s="137" t="n"/>
@@ -6960,7 +6960,7 @@
       </c>
       <c r="F150" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Ürünleri kriter bazında yan yana gösteren standart karşılaştırma tablosu şablonu hazırlanır.</t>
         </is>
       </c>
       <c r="G150" s="137" t="n"/>
@@ -6994,7 +6994,7 @@
       </c>
       <c r="F151" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Her tablo için kullanıcı kararını etkileyen en az 5-7 ayırt edici kriter belirlenir.</t>
         </is>
       </c>
       <c r="G151" s="137" t="n"/>
@@ -7028,7 +7028,7 @@
       </c>
       <c r="F152" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Karşılaştırma tabloları ilgili kategori ve ürün sayfalarına yerleştirilir.</t>
         </is>
       </c>
       <c r="G152" s="137" t="n"/>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="F155" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Her kategori için müşteri sorularını yanıtlayan SSS içerikleri yazılır.</t>
         </is>
       </c>
       <c r="G155" s="137" t="n"/>
@@ -7180,7 +7180,7 @@
       </c>
       <c r="F156" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Kargo, iade, ödeme ve teslimat gibi satın alma sürecine dair soruları yanıtlayan SSS sayfası hazırlanır.</t>
         </is>
       </c>
       <c r="G156" s="137" t="n"/>
@@ -7214,7 +7214,7 @@
       </c>
       <c r="F157" s="137" t="inlineStr">
         <is>
-          <t>Action'lar implement edilmeliydi, sonuçlar measured edilmeliydi.</t>
+          <t>Oluşturulan SSS içerikleri FAQPage schema ile işaretlenir.</t>
         </is>
       </c>
       <c r="G157" s="137" t="n"/>
@@ -7332,7 +7332,7 @@
       </c>
       <c r="F160" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Karar aşamasında rehbere en çok ihtiyaç duyulan kategoriler trafik ve dönüşüm potansiyeline göre önceliklendirilir.</t>
         </is>
       </c>
       <c r="G160" s="137" t="n"/>
@@ -7366,7 +7366,7 @@
       </c>
       <c r="F161" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Giriş, seçim kriterleri, öneriler ve SSS bölümlerini içeren alıcı rehberi şablonu hazırlanır.</t>
         </is>
       </c>
       <c r="G161" s="137" t="n"/>
@@ -7434,7 +7434,7 @@
       </c>
       <c r="F163" s="137" t="inlineStr">
         <is>
-          <t>Action'lar implement edilmeliydi, sonuçlar measured edilmeliydi.</t>
+          <t>Adımlı rehber içeriklerine HowTo schema uygulanır.</t>
         </is>
       </c>
       <c r="G163" s="137" t="n"/>
@@ -7552,7 +7552,7 @@
       </c>
       <c r="F166" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>İçeriklerde sayı, oran ve tarihlerin kaynağıyla birlikte verilmesini sağlayan atıf standardı belirlenir.</t>
         </is>
       </c>
       <c r="G166" s="137" t="n"/>
@@ -7586,7 +7586,7 @@
       </c>
       <c r="F167" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Mevcut içeriklerde iddia içeren ancak kaynak gösterilmeyen bölümler taranır.</t>
         </is>
       </c>
       <c r="G167" s="137" t="n"/>
@@ -7620,7 +7620,7 @@
       </c>
       <c r="F168" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Tespit edilen bölümlere güncel istatistik ve güvenilir kaynak referansları eklenir.</t>
         </is>
       </c>
       <c r="G168" s="137" t="n"/>
@@ -7654,7 +7654,7 @@
       </c>
       <c r="F169" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>GEO açısından kritik sayfalara görünür 'son güncelleme' tarihi eklenerek içerik tazeliği sinyali verilir.</t>
         </is>
       </c>
       <c r="G169" s="137" t="n"/>
@@ -7806,7 +7806,7 @@
       </c>
       <c r="F173" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Uygun başlıklar kullanıcı sorgularıyla eşleşecek soru formatına dönüştürülerek AI yanıtlarında eşleşme artırılır.</t>
         </is>
       </c>
       <c r="G173" s="137" t="n"/>
@@ -7840,7 +7840,7 @@
       </c>
       <c r="F174" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Her bölümün ilk cümlesi, bağlamdan bağımsız anlaşılır ve alıntılanabilir şekilde yazılır.</t>
         </is>
       </c>
       <c r="G174" s="137" t="n"/>
@@ -7874,7 +7874,7 @@
       </c>
       <c r="F175" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>İçerik, AI'ın kolay ayrıştırabilmesi için kısa paragraflar, başlıklar ve listelerle parçalanabilir hale getirilir.</t>
         </is>
       </c>
       <c r="G175" s="137" t="n"/>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="F177" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Marka, ürün grupları ve kategoriler gibi ana entity'ler ve aralarındaki ilişkiler haritalanır.</t>
         </is>
       </c>
       <c r="G177" s="137" t="n"/>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="F178" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Her ana entity için kapsamlı bir pillar sayfası belirlenir veya planlanır.</t>
         </is>
       </c>
       <c r="G178" s="137" t="n"/>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="F179" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Pillar sayfaları destekleyen alt konu (cluster) içerik planı oluşturulur.</t>
         </is>
       </c>
       <c r="G179" s="137" t="n"/>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="F181" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Ana entity'ler ilgili schema türleriyle işaretlenerek anlamsal netlik güçlendirilir.</t>
         </is>
       </c>
       <c r="G181" s="137" t="n"/>
@@ -8178,7 +8178,7 @@
       </c>
       <c r="F183" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>GSC'den düşük rekabetli, niyet odaklı long-tail sorgular çekilerek içerik fırsatları belirlenir.</t>
         </is>
       </c>
       <c r="G183" s="137" t="n"/>
@@ -8280,7 +8280,7 @@
       </c>
       <c r="F186" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>İçeriklere kullanıcıların doğal dildeki sorularını karşılayan soru formatlı başlıklar eklenir.</t>
         </is>
       </c>
       <c r="G186" s="137" t="n"/>
@@ -8466,7 +8466,7 @@
       </c>
       <c r="F191" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>AI yanıtlarında sürekli atıflanan site türleri tespit edilerek backlink stratejisine yön verilir.</t>
         </is>
       </c>
       <c r="G191" s="137" t="n"/>
@@ -8500,7 +8500,7 @@
       </c>
       <c r="F192" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Atıf potansiyeli yüksek siteler önceliklendirilerek backlink hedef listesi oluşturulur.</t>
         </is>
       </c>
       <c r="G192" s="137" t="n"/>
@@ -8584,7 +8584,7 @@
       </c>
       <c r="F194" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Hedef kitlenin aktif olduğu subreddit ve forumlar belirlenir.</t>
         </is>
       </c>
       <c r="G194" s="137" t="n"/>
@@ -8618,7 +8618,7 @@
       </c>
       <c r="F195" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Topluluklarda en sık sorulan sorular temalara göre gruplanır.</t>
         </is>
       </c>
       <c r="G195" s="137" t="n"/>
@@ -8652,7 +8652,7 @@
       </c>
       <c r="F196" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Yanıtsız veya zayıf yanıtlanan sorular içerik fırsatı olarak işaretlenir.</t>
         </is>
       </c>
       <c r="G196" s="137" t="n"/>
@@ -8686,7 +8686,7 @@
       </c>
       <c r="F197" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Belirlenen sorular içerik takvimine eklenerek planlı şekilde yanıtlanır.</t>
         </is>
       </c>
       <c r="G197" s="137" t="n"/>
@@ -9178,7 +9178,7 @@
       </c>
       <c r="F211" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Marka, ürün ve kategorilere dayalı temel (seed) anahtar kelime listesi oluşturulur.</t>
         </is>
       </c>
       <c r="G211" s="137" t="n"/>
@@ -9212,7 +9212,7 @@
       </c>
       <c r="F212" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Seed kelimeler Ahrefs/SEOMonitor ile genişletilerek hacim ve zorluk verisiyle zenginleştirilir.</t>
         </is>
       </c>
       <c r="G212" s="137" t="n"/>
@@ -9314,7 +9314,7 @@
       </c>
       <c r="F215" s="137" t="inlineStr">
         <is>
-          <t>İçerik publish edilmeliydi, indexing beklenmeliydi.</t>
+          <t>Konu haritası yayın takvimiyle eşleştirilerek her dönemde hangi içeriğin üretileceği planlanır.</t>
         </is>
       </c>
       <c r="G215" s="137" t="n"/>
@@ -9398,7 +9398,7 @@
       </c>
       <c r="F217" s="137" t="inlineStr">
         <is>
-          <t>İçerik publish edilmeliydi, indexing beklenmeliydi.</t>
+          <t>Ekip kapasitesine göre sürdürülebilir bir yayın sıklığı (haftalık/iki haftalık) belirlenir.</t>
         </is>
       </c>
       <c r="G217" s="137" t="n"/>
@@ -9432,7 +9432,7 @@
       </c>
       <c r="F218" s="137" t="inlineStr">
         <is>
-          <t>Veri analiz yapılmalı, insight'lar çıkarılmalıydı.</t>
+          <t>How-to, rehber, karşılaştırma ve trend analizi gibi içerik türlerinin dengeli dağılımı planlanır.</t>
         </is>
       </c>
       <c r="G218" s="137" t="n"/>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="F219" s="137" t="inlineStr">
         <is>
-          <t>Sistem veya tool entegrasyonu yapılmalıydı.</t>
+          <t>Brief, yazım, review, schema ve yayın adımlarını içeren editoryal iş akışı kurulur.</t>
         </is>
       </c>
       <c r="G219" s="137" t="n"/>
@@ -9500,7 +9500,7 @@
       </c>
       <c r="F220" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Mevcut içeriklerin düzenli güncellenmesi için tazelik (freshness) takvimi oluşturulur.</t>
         </is>
       </c>
       <c r="G220" s="137" t="n"/>
@@ -9618,7 +9618,7 @@
       </c>
       <c r="F223" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Tutarlı numaralı adımlar, görseller ve özet içeren how-to içerik şablonu hazırlanır.</t>
         </is>
       </c>
       <c r="G223" s="137" t="n"/>
@@ -9652,7 +9652,7 @@
       </c>
       <c r="F224" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Her rehbere anlatımı destekleyen özgün görsel veya infografik eklenir.</t>
         </is>
       </c>
       <c r="G224" s="137" t="n"/>
@@ -9686,7 +9686,7 @@
       </c>
       <c r="F225" s="137" t="inlineStr">
         <is>
-          <t>Action'lar implement edilmeliydi, sonuçlar measured edilmeliydi.</t>
+          <t>Adımlı rehberlere HowTo schema uygulanır.</t>
         </is>
       </c>
       <c r="G225" s="137" t="n"/>
@@ -9770,7 +9770,7 @@
       </c>
       <c r="F227" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>İçeriklerin çeyreklik olarak gözden geçirileceği güncelleme takvimi oluşturulur.</t>
         </is>
       </c>
       <c r="G227" s="137" t="n"/>
@@ -9804,7 +9804,7 @@
       </c>
       <c r="F228" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Trafik kaybeden içerikler tespit edilerek güncelleme önceliği verilir.</t>
         </is>
       </c>
       <c r="G228" s="137" t="n"/>
@@ -9838,7 +9838,7 @@
       </c>
       <c r="F229" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>İçeriklere güncel istatistik, veri ve yeni gelişmeler eklenerek tazelik sağlanır.</t>
         </is>
       </c>
       <c r="G229" s="137" t="n"/>
@@ -9956,7 +9956,7 @@
       </c>
       <c r="F232" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Özgün araştırmanın konusu, veri kaynağı ve metodolojisi netleştirilir.</t>
         </is>
       </c>
       <c r="G232" s="137" t="n"/>
@@ -10024,7 +10024,7 @@
       </c>
       <c r="F234" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Araştırma bulguları görsellerle desteklenmiş bir rapor olarak yayınlanır.</t>
         </is>
       </c>
       <c r="G234" s="137" t="n"/>
@@ -10058,7 +10058,7 @@
       </c>
       <c r="F235" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Araştırma sonuçları basın bülteniyle duyurularak atıf ve backlink potansiyeli oluşturulur.</t>
         </is>
       </c>
       <c r="G235" s="137" t="n"/>
@@ -10142,7 +10142,7 @@
       </c>
       <c r="F237" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>İçeriklerde kaynak gösterimi için tutarlı bir atıf standardı belirlenir.</t>
         </is>
       </c>
       <c r="G237" s="137" t="n"/>
@@ -10176,7 +10176,7 @@
       </c>
       <c r="F238" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Her blog yazısına konuyu destekleyen en az 3-5 güvenilir kaynak referansı eklenir.</t>
         </is>
       </c>
       <c r="G238" s="137" t="n"/>
@@ -10210,7 +10210,7 @@
       </c>
       <c r="F239" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>İstatistiklerde kaynak, tarih ve kapsam (popülasyon) bilgisi belirtilir.</t>
         </is>
       </c>
       <c r="G239" s="137" t="n"/>
@@ -10244,7 +10244,7 @@
       </c>
       <c r="F240" s="137" t="inlineStr">
         <is>
-          <t>İlgili alan doğruluk için review edilmeliydi.</t>
+          <t>Editoryal kontrol listesine kaynak ve atıf doğrulama adımı eklenir.</t>
         </is>
       </c>
       <c r="G240" s="137" t="n"/>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="F243" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Varsa mevcut Wikipedia sayfası içerik ve kaynak açısından incelenir.</t>
         </is>
       </c>
       <c r="G243" s="137" t="n"/>
@@ -10380,7 +10380,7 @@
       </c>
       <c r="F244" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Sayfadaki eksik veya güncel olmayan bilgiler tespit edilir.</t>
         </is>
       </c>
       <c r="G244" s="137" t="n"/>
@@ -10414,7 +10414,7 @@
       </c>
       <c r="F245" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Güncellemeler güvenilir, bağımsız kaynaklarla desteklenerek tarafsız üslupla yapılır.</t>
         </is>
       </c>
       <c r="G245" s="137" t="n"/>
@@ -10448,7 +10448,7 @@
       </c>
       <c r="F246" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Markanın Wikipedia notability (kayda değerlik) kriterlerini karşılayıp karşılamadığı değerlendirilir.</t>
         </is>
       </c>
       <c r="G246" s="137" t="n"/>
@@ -10482,7 +10482,7 @@
       </c>
       <c r="F247" s="137" t="inlineStr">
         <is>
-          <t>Metric'ler regular olarak monitor edilmeliydi.</t>
+          <t>Düzenlemeler Wikipedia'nın tarafsızlık ve kaynak politikalarına uygun şekilde yapılır.</t>
         </is>
       </c>
       <c r="G247" s="137" t="n"/>
@@ -10566,7 +10566,7 @@
       </c>
       <c r="F249" s="137" t="inlineStr">
         <is>
-          <t>İlgili alan doğruluk için review edilmeliydi.</t>
+          <t>Tüm Google Business profilleri kategori, çalışma saati, foto ve açıklama açısından eksiksiz doldurulur.</t>
         </is>
       </c>
       <c r="G249" s="137" t="n"/>
@@ -10634,7 +10634,7 @@
       </c>
       <c r="F251" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Düzenli güncellik için haftalık GBP gönderi takvimi oluşturulur.</t>
         </is>
       </c>
       <c r="G251" s="137" t="n"/>
@@ -10668,7 +10668,7 @@
       </c>
       <c r="F252" s="137" t="inlineStr">
         <is>
-          <t>Sistem veya tool entegrasyonu yapılmalıydı.</t>
+          <t>Gelen yorumların belirli sürede yanıtlanması için bir süreç tanımlanır.</t>
         </is>
       </c>
       <c r="G252" s="137" t="n"/>
@@ -10702,7 +10702,7 @@
       </c>
       <c r="F253" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>GBP soru-cevap bölümü sık sorulan sorularla proaktif olarak doldurulur.</t>
         </is>
       </c>
       <c r="G253" s="137" t="n"/>
@@ -10786,7 +10786,7 @@
       </c>
       <c r="F255" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Mevcut şikayetler analiz edilip tema ve kök nedenlerine göre kategorize edilir.</t>
         </is>
       </c>
       <c r="G255" s="137" t="n"/>
@@ -10820,7 +10820,7 @@
       </c>
       <c r="F256" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Yanıtlanmamış şikayetler çözüm odaklı şekilde yanıtlanır.</t>
         </is>
       </c>
       <c r="G256" s="137" t="n"/>
@@ -10854,7 +10854,7 @@
       </c>
       <c r="F257" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Sık karşılaşılan durumlar için çözüm odaklı yanıt şablonları hazırlanır.</t>
         </is>
       </c>
       <c r="G257" s="137" t="n"/>
@@ -10888,7 +10888,7 @@
       </c>
       <c r="F258" s="137" t="inlineStr">
         <is>
-          <t>Sistem veya tool entegrasyonu yapılmalıydı.</t>
+          <t>Yeni şikayetlerin düzenli izlenmesi için haftalık takip süreci kurulur.</t>
         </is>
       </c>
       <c r="G258" s="137" t="n"/>
@@ -11006,7 +11006,7 @@
       </c>
       <c r="F261" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Trustpilot, Google ve diğer platformlardaki mevcut puan ve yorum durumu raporlanır.</t>
         </is>
       </c>
       <c r="G261" s="137" t="n"/>
@@ -11040,7 +11040,7 @@
       </c>
       <c r="F262" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Satış sonrası e-posta akışıyla memnun müşterilerden yorum toplama stratejisi kurulur.</t>
         </is>
       </c>
       <c r="G262" s="137" t="n"/>
@@ -11074,7 +11074,7 @@
       </c>
       <c r="F263" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Olumsuz yorumlara 24-48 saat içinde çözüm odaklı yanıt verilir.</t>
         </is>
       </c>
       <c r="G263" s="137" t="n"/>
@@ -11108,7 +11108,7 @@
       </c>
       <c r="F264" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Yorum hacmi, ortalama puan ve tema dağılımı aylık raporlanır.</t>
         </is>
       </c>
       <c r="G264" s="137" t="n"/>
@@ -11192,7 +11192,7 @@
       </c>
       <c r="F266" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>G2/Capterra profili açıklama, özellik ve görsellerle eksiksiz doldurulur.</t>
         </is>
       </c>
       <c r="G266" s="137" t="n"/>
@@ -11260,7 +11260,7 @@
       </c>
       <c r="F268" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Ürün/hizmet bilgileri ve fiyatlandırma profilde güncel tutulur.</t>
         </is>
       </c>
       <c r="G268" s="137" t="n"/>
@@ -11344,7 +11344,7 @@
       </c>
       <c r="F270" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Markayla ilgili konuların tartışıldığı subreddit'ler belirlenir.</t>
         </is>
       </c>
       <c r="G270" s="137" t="n"/>
@@ -11412,7 +11412,7 @@
       </c>
       <c r="F272" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Spam algısı yaratmadan düzenli katılım için haftalık plan oluşturulur.</t>
         </is>
       </c>
       <c r="G272" s="137" t="n"/>
@@ -11446,7 +11446,7 @@
       </c>
       <c r="F273" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Sorulara satış odaklı olmayan, gerçekten değer katan yanıtlar verilir.</t>
         </is>
       </c>
       <c r="G273" s="137" t="n"/>
@@ -11564,7 +11564,7 @@
       </c>
       <c r="F276" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Hedef kitlenin ilgi alanlarına göre düzenli video içerik takvimi oluşturulur.</t>
         </is>
       </c>
       <c r="G276" s="137" t="n"/>
@@ -11598,7 +11598,7 @@
       </c>
       <c r="F277" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Giriş, içerik ve CTA bölümlerini içeren tutarlı video şablonu hazırlanır.</t>
         </is>
       </c>
       <c r="G277" s="137" t="n"/>
@@ -11632,7 +11632,7 @@
       </c>
       <c r="F278" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Başlık, açıklama, etiket ve chapter'lar arama ve öneri için optimize edilir.</t>
         </is>
       </c>
       <c r="G278" s="137" t="n"/>
@@ -11666,7 +11666,7 @@
       </c>
       <c r="F279" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Video açıklamalarına ilgili site sayfalarına yönlendiren linkler eklenir.</t>
         </is>
       </c>
       <c r="G279" s="137" t="n"/>
@@ -11700,7 +11700,7 @@
       </c>
       <c r="F280" s="137" t="inlineStr">
         <is>
-          <t>İçerik publish edilmeliydi, indexing beklenmeliydi.</t>
+          <t>Video transcript'leri düzenlenerek blog içeriği olarak yayınlanır ve içerik yeniden değerlendirilir.</t>
         </is>
       </c>
       <c r="G280" s="137" t="n"/>
@@ -11818,7 +11818,7 @@
       </c>
       <c r="F283" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Veri ve hikaye açılarına dayalı aylık dijital PR takvimi hazırlanır.</t>
         </is>
       </c>
       <c r="G283" s="137" t="n"/>
@@ -11886,7 +11886,7 @@
       </c>
       <c r="F285" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Uzman görüşü ve özgün veriye dayalı, basının ilgisini çekecek hikaye açıları belirlenir.</t>
         </is>
       </c>
       <c r="G285" s="137" t="n"/>
@@ -11920,7 +11920,7 @@
       </c>
       <c r="F286" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Yayınların AI yanıtlarındaki marka atıflarına etkisi ölçülür.</t>
         </is>
       </c>
       <c r="G286" s="137" t="n"/>
@@ -12004,7 +12004,7 @@
       </c>
       <c r="F288" s="137" t="inlineStr">
         <is>
-          <t>Veri analiz yapılmalı, insight'lar çıkarılmalıydı.</t>
+          <t>Query Fan-Out analizinden AI'ın sık atıfladığı siteler guest post hedefi olarak belirlenir.</t>
         </is>
       </c>
       <c r="G288" s="137" t="n"/>
@@ -12038,7 +12038,7 @@
       </c>
       <c r="F289" s="137" t="inlineStr">
         <is>
-          <t>İlgili alan doğruluk için review edilmeliydi.</t>
+          <t>Konuk yazı kabul eden siteler DA/DR ve konu uyumu açısından değerlendirilerek listelenir.</t>
         </is>
       </c>
       <c r="G289" s="137" t="n"/>
@@ -12072,7 +12072,7 @@
       </c>
       <c r="F290" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Her hedef site için konuya ve kitleye uygun konu önerisi ve pitch hazırlanır.</t>
         </is>
       </c>
       <c r="G290" s="137" t="n"/>
@@ -12106,7 +12106,7 @@
       </c>
       <c r="F291" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Yazılar markayı doğal ve değer katan bir bağlamda içerecek şekilde kurgulanır.</t>
         </is>
       </c>
       <c r="G291" s="137" t="n"/>
@@ -12140,7 +12140,7 @@
       </c>
       <c r="F292" s="137" t="inlineStr">
         <is>
-          <t>İçerik publish edilmeliydi, indexing beklenmeliydi.</t>
+          <t>Yayınlanan yazıların marka görünürlüğüne ve AI atıflarına etkisi takip edilir.</t>
         </is>
       </c>
       <c r="G292" s="137" t="n"/>
@@ -12224,7 +12224,7 @@
       </c>
       <c r="F294" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Sektörle ilgili haber siteleri ve yayınlardan oluşan medya listesi oluşturulur.</t>
         </is>
       </c>
       <c r="G294" s="137" t="n"/>
@@ -12258,7 +12258,7 @@
       </c>
       <c r="F295" s="137" t="inlineStr">
         <is>
-          <t>Metric'ler regular olarak monitor edilmeliydi.</t>
+          <t>Uzman görüşü ve röportaj fırsatları düzenli olarak takip edilir.</t>
         </is>
       </c>
       <c r="G295" s="137" t="n"/>
@@ -12292,7 +12292,7 @@
       </c>
       <c r="F296" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Otorite sitelerde sponsorlu içerik olanakları değerlendirilir.</t>
         </is>
       </c>
       <c r="G296" s="137" t="n"/>
@@ -12444,7 +12444,7 @@
       </c>
       <c r="F300" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Sosyal medya paylaşımlarında tutarlı marka mesajı ve hedef anahtar kelimeler kullanılır.</t>
         </is>
       </c>
       <c r="G300" s="137" t="n"/>
@@ -12512,7 +12512,7 @@
       </c>
       <c r="F302" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Kullanıcı üretimi içeriği (UGC) teşvik eden ve toplayan bir strateji oluşturulur.</t>
         </is>
       </c>
       <c r="G302" s="137" t="n"/>
@@ -12664,7 +12664,7 @@
       </c>
       <c r="F306" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Yöneticiler için haftalık, derinlemesine sektörel paylaşım planı oluşturulur.</t>
         </is>
       </c>
       <c r="G306" s="137" t="n"/>
@@ -12698,7 +12698,7 @@
       </c>
       <c r="F307" s="137" t="inlineStr">
         <is>
-          <t>İçerik publish edilmeliydi, indexing beklenmeliydi.</t>
+          <t>Uzmanlık gösteren özgün LinkedIn makaleleri düzenli olarak yayınlanır.</t>
         </is>
       </c>
       <c r="G307" s="137" t="n"/>
@@ -12850,7 +12850,7 @@
       </c>
       <c r="F311" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Dizinlerdeki ad, adres ve telefon (NAP) tutarsızlıkları tespit edilip düzeltilir.</t>
         </is>
       </c>
       <c r="G311" s="137" t="n"/>
@@ -12884,7 +12884,7 @@
       </c>
       <c r="F312" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Eksik olan ilgili dizinlere tutarlı NAP bilgisiyle yeni kayıtlar yapılır.</t>
         </is>
       </c>
       <c r="G312" s="137" t="n"/>
@@ -12986,7 +12986,7 @@
       </c>
       <c r="F315" s="137" t="inlineStr">
         <is>
-          <t>Mevcut durum kontrol edilmeliydi.</t>
+          <t>Mevcut listelerdeki eksik işletme bilgileri tamamlanır.</t>
         </is>
       </c>
       <c r="G315" s="137" t="n"/>
@@ -13020,7 +13020,7 @@
       </c>
       <c r="F316" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Yeni dizin ve liste fırsatları düzenli olarak takip edilir.</t>
         </is>
       </c>
       <c r="G316" s="137" t="n"/>
@@ -13104,7 +13104,7 @@
       </c>
       <c r="F318" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Yandex Webmaster Tools hesabı oluşturulur.</t>
         </is>
       </c>
       <c r="G318" s="137" t="n"/>
@@ -13138,7 +13138,7 @@
       </c>
       <c r="F319" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Site sahipliği Yandex Webmaster Tools üzerinden doğrulanır.</t>
         </is>
       </c>
       <c r="G319" s="137" t="n"/>
@@ -13172,7 +13172,7 @@
       </c>
       <c r="F320" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>XML sitemap Yandex'e gönderilerek indexleme başlatılır.</t>
         </is>
       </c>
       <c r="G320" s="137" t="n"/>
@@ -13206,7 +13206,7 @@
       </c>
       <c r="F321" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>İşletme Yandex Business Directory'ye kaydedilir.</t>
         </is>
       </c>
       <c r="G321" s="137" t="n"/>
@@ -13240,7 +13240,7 @@
       </c>
       <c r="F322" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Yandex Reviews'da işletme profili oluşturularak yorum yönetimi başlatılır.</t>
         </is>
       </c>
       <c r="G322" s="137" t="n"/>
@@ -13342,7 +13342,7 @@
       </c>
       <c r="F325" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Tutarlı yazar profil sayfaları için biyografi, uzmanlık ve görsel içeren şablon hazırlanır.</t>
         </is>
       </c>
       <c r="G325" s="137" t="n"/>
@@ -13376,7 +13376,7 @@
       </c>
       <c r="F326" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Her yazara biyografi, uzmanlık alanı ve sosyal medya bağlantıları eklenir.</t>
         </is>
       </c>
       <c r="G326" s="137" t="n"/>
@@ -13410,7 +13410,7 @@
       </c>
       <c r="F327" s="137" t="inlineStr">
         <is>
-          <t>Action'lar implement edilmeliydi, sonuçlar measured edilmeliydi.</t>
+          <t>Yazar profillerine Person (JSON-LD) schema uygulanır.</t>
         </is>
       </c>
       <c r="G327" s="137" t="n"/>
@@ -13444,7 +13444,7 @@
       </c>
       <c r="F328" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Blog yazıları yazar profil sayfasına bağlanarak E-E-A-T sinyali güçlendirilir.</t>
         </is>
       </c>
       <c r="G328" s="137" t="n"/>
@@ -13528,7 +13528,7 @@
       </c>
       <c r="F330" s="137" t="inlineStr">
         <is>
-          <t>İlgili bilgi veya element eklenmeliydi.</t>
+          <t>Hakkımızda sayfasına ekip ve uzmanları tanıtan bir bölüm eklenir.</t>
         </is>
       </c>
       <c r="G330" s="137" t="n"/>
@@ -13562,7 +13562,7 @@
       </c>
       <c r="F331" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>İletişim sayfası adres, telefon, e-posta ve harita ile detaylandırılır.</t>
         </is>
       </c>
       <c r="G331" s="137" t="n"/>
@@ -13680,7 +13680,7 @@
       </c>
       <c r="F334" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Bing Merchant Center hesabı açılır.</t>
         </is>
       </c>
       <c r="G334" s="137" t="n"/>
@@ -13714,7 +13714,7 @@
       </c>
       <c r="F335" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Ürün feed'i oluşturulup Bing Merchant Center'a gönderilir.</t>
         </is>
       </c>
       <c r="G335" s="137" t="n"/>
@@ -13748,7 +13748,7 @@
       </c>
       <c r="F336" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Feed'deki eksik alan ve hatalar giderilerek onay oranı yükseltilir.</t>
         </is>
       </c>
       <c r="G336" s="137" t="n"/>
@@ -14782,7 +14782,7 @@
       </c>
       <c r="F365" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Düzenli infografik üretimi için içerik takvimi oluşturulur.</t>
         </is>
       </c>
       <c r="G365" s="137" t="n"/>
@@ -14850,7 +14850,7 @@
       </c>
       <c r="F367" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Sürdürülebilir video içerik üretimi için bir süreç başlatılır.</t>
         </is>
       </c>
       <c r="G367" s="137" t="n"/>
@@ -14884,7 +14884,7 @@
       </c>
       <c r="F368" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Görsel alt text ve caption'lar hedef anahtar kelimelerle ve betimleyici şekilde yazılır.</t>
         </is>
       </c>
       <c r="G368" s="137" t="n"/>
@@ -14968,7 +14968,7 @@
       </c>
       <c r="F370" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Marka ve kitleyle uyumlu hedef influencer listesi oluşturulur.</t>
         </is>
       </c>
       <c r="G370" s="137" t="n"/>
@@ -15002,7 +15002,7 @@
       </c>
       <c r="F371" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Review, ortak üretim veya sponsorluk gibi iş birliği modelleri belirlenir.</t>
         </is>
       </c>
       <c r="G371" s="137" t="n"/>
@@ -15036,7 +15036,7 @@
       </c>
       <c r="F372" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Influencer içeriklerinde markanın doğal şekilde anılması sağlanır.</t>
         </is>
       </c>
       <c r="G372" s="137" t="n"/>
@@ -15070,7 +15070,7 @@
       </c>
       <c r="F373" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>İş birliklerinin marka görünürlüğüne ve AI atıflarına etkisi ölçülür.</t>
         </is>
       </c>
       <c r="G373" s="137" t="n"/>
@@ -15154,7 +15154,7 @@
       </c>
       <c r="F375" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>AI platformlarındaki yeni sorgu ve konu trendleri düzenli olarak izlenir.</t>
         </is>
       </c>
       <c r="G375" s="137" t="n"/>
@@ -15188,7 +15188,7 @@
       </c>
       <c r="F376" s="137" t="inlineStr">
         <is>
-          <t>Sistem veya tool entegrasyonu yapılmalıydı.</t>
+          <t>Yükselen konularda hızlı içerik üretimi için çevik bir süreç kurulur.</t>
         </is>
       </c>
       <c r="G376" s="137" t="n"/>
@@ -15222,7 +15222,7 @@
       </c>
       <c r="F377" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Sezonsal talep dönemleri için içerik önceden planlanır.</t>
         </is>
       </c>
       <c r="G377" s="137" t="n"/>
@@ -15256,7 +15256,7 @@
       </c>
       <c r="F378" s="137" t="inlineStr">
         <is>
-          <t>Sistem veya tool entegrasyonu yapılmalıydı.</t>
+          <t>Yükselen aramaları izleyen bir dashboard kurularak fırsatlar erken yakalanır.</t>
         </is>
       </c>
       <c r="G378" s="137" t="n"/>
@@ -15340,7 +15340,7 @@
       </c>
       <c r="F380" s="137" t="inlineStr">
         <is>
-          <t>Sistem veya tool entegrasyonu yapılmalıydı.</t>
+          <t>Schema hatalarını otomatik tespit eden bir doğrulama script'i kurulur.</t>
         </is>
       </c>
       <c r="G380" s="137" t="n"/>
@@ -15374,7 +15374,7 @@
       </c>
       <c r="F381" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>İçerik tazeliği düştüğünde uyarı veren bir alert sistemi kurulur.</t>
         </is>
       </c>
       <c r="G381" s="137" t="n"/>
@@ -15408,7 +15408,7 @@
       </c>
       <c r="F382" s="137" t="inlineStr">
         <is>
-          <t>Sistem veya tool entegrasyonu yapılmalıydı.</t>
+          <t>AI bot crawl aktivitesindeki anormallikler için uyarı sistemi kurulur.</t>
         </is>
       </c>
       <c r="G382" s="137" t="n"/>
@@ -15442,7 +15442,7 @@
       </c>
       <c r="F383" s="137" t="inlineStr">
         <is>
-          <t>Sistem veya tool entegrasyonu yapılmalıydı.</t>
+          <t>Kırık link ve 404'leri otomatik tespit eden bir sistem kurulur.</t>
         </is>
       </c>
       <c r="G383" s="137" t="n"/>
@@ -15526,7 +15526,7 @@
       </c>
       <c r="F385" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Agentic commerce trendleri ve gereksinimleri araştırılarak yol haritası çıkarılır.</t>
         </is>
       </c>
       <c r="G385" s="137" t="n"/>
@@ -15560,7 +15560,7 @@
       </c>
       <c r="F386" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Ürün kataloğu yapısal ve API erişimine hazır hale getirilir.</t>
         </is>
       </c>
       <c r="G386" s="137" t="n"/>
@@ -15628,7 +15628,7 @@
       </c>
       <c r="F388" s="137" t="inlineStr">
         <is>
-          <t>Metric'ler regular olarak monitor edilmeliydi.</t>
+          <t>ChatGPT Shopping gibi entegrasyon fırsatları takip edilerek erken uyum sağlanır.</t>
         </is>
       </c>
       <c r="G388" s="137" t="n"/>
@@ -15748,7 +15748,7 @@
       </c>
       <c r="F392" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Metrikler önceki ayla karşılaştırılarak ilerleme ve gerilemeler ortaya konur.</t>
         </is>
       </c>
       <c r="G392" s="137" t="n"/>
@@ -15782,7 +15782,7 @@
       </c>
       <c r="F393" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Rapor bulgularına dayalı somut aksiyon önerileri yazılır.</t>
         </is>
       </c>
       <c r="G393" s="137" t="n"/>
@@ -15866,7 +15866,7 @@
       </c>
       <c r="F395" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Belirlenen takip sorguları haftalık olarak AI platformlarında çalıştırılır.</t>
         </is>
       </c>
       <c r="G395" s="137" t="n"/>
@@ -15900,7 +15900,7 @@
       </c>
       <c r="F396" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Yeni kazanılan ve kaybedilen marka atıfları tespit edilir.</t>
         </is>
       </c>
       <c r="G396" s="137" t="n"/>
@@ -15968,7 +15968,7 @@
       </c>
       <c r="F398" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Atıf durumu ve önemli değişiklikler haftalık özet raporda toplanır.</t>
         </is>
       </c>
       <c r="G398" s="137" t="n"/>
@@ -16086,7 +16086,7 @@
       </c>
       <c r="F401" s="137" t="inlineStr">
         <is>
-          <t>Gereken aksiyon uygulanmalıydı.</t>
+          <t>Rakiplere karşı Share of Voice'un zaman içindeki trendi analiz edilir.</t>
         </is>
       </c>
       <c r="G401" s="137" t="n"/>
@@ -16154,7 +16154,7 @@
       </c>
       <c r="F403" s="137" t="inlineStr">
         <is>
-          <t>Veri analiz yapılmalı, insight'lar çıkarılmalıydı.</t>
+          <t>Rakip karşısındaki içerik ve atıf boşlukları güncellenerek yeni fırsatlar belirlenir.</t>
         </is>
       </c>
       <c r="G403" s="137" t="n"/>
@@ -16238,7 +16238,7 @@
       </c>
       <c r="F405" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Marka algısını ölçmek için sentiment analiz yöntemi ve kaynakları belirlenir.</t>
         </is>
       </c>
       <c r="G405" s="137" t="n"/>
@@ -16306,7 +16306,7 @@
       </c>
       <c r="F407" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Olumsuz algıyı tetikleyen konular ve kaynaklar tespit edilir.</t>
         </is>
       </c>
       <c r="G407" s="137" t="n"/>
@@ -16340,7 +16340,7 @@
       </c>
       <c r="F408" s="137" t="inlineStr">
         <is>
-          <t>Yeni bir sistem veya liste oluşturulmalıydı.</t>
+          <t>Olumsuz algıyı gidermeye yönelik düzeltici aksiyon planı oluşturulur.</t>
         </is>
       </c>
       <c r="G408" s="137" t="n"/>
@@ -16458,7 +16458,7 @@
       </c>
       <c r="F411" s="137" t="inlineStr">
         <is>
-          <t>Bu sub-step execute edilmeli, sonuçlar main task'ın completion'ı için critical'dır.</t>
+          <t>Geçersiz veya eksik schema işaretlemeleri tespit edilip düzeltilir.</t>
         </is>
       </c>
       <c r="G411" s="137" t="n"/>
@@ -16492,7 +16492,7 @@
       </c>
       <c r="F412" s="137" t="inlineStr">
         <is>
-          <t>İlgili alan doğruluk için review edilmeliydi.</t>
+          <t>İçeriklerin güncelliği gözden geçirilerek tazelik gerektiren sayfalar belirlenir.</t>
         </is>
       </c>
       <c r="G412" s="137" t="n"/>
@@ -16560,7 +16560,7 @@
       </c>
       <c r="F414" s="137" t="inlineStr">
         <is>
-          <t>Plan, template veya dokümantasyon oluşturulmalıydı.</t>
+          <t>Denetim bulguları raporlanarak önceliklendirilmiş bir aksiyon listesi çıkarılır.</t>
         </is>
       </c>
       <c r="G414" s="137" t="n"/>

</xml_diff>